<commit_message>
Inverted Logic on Toggle Switches
</commit_message>
<xml_diff>
--- a/docs/Stations/Station_Wiring_FR.xlsx
+++ b/docs/Stations/Station_Wiring_FR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/My Files/EDCQ/Projects/Controls/Cabane Controls/Package 2/Arduino/docs/Stations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565CFA0F-2FF2-E243-B3C3-F53EBFCEF354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81BC5926-D33D-EA41-88AA-794A1AEB677F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>ST3</t>
   </si>
   <si>
-    <t>ST4</t>
-  </si>
-  <si>
     <t>ST5</t>
   </si>
   <si>
@@ -270,6 +267,9 @@
   </si>
   <si>
     <t>Jaune / Rouge</t>
+  </si>
+  <si>
+    <t>ST4 - ST5</t>
   </si>
 </sst>
 </file>
@@ -882,7 +882,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>1</v>
@@ -900,16 +900,16 @@
         <v>5</v>
       </c>
       <c r="H1" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="I1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="K1" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -917,34 +917,34 @@
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>11</v>
-      </c>
       <c r="D2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="G2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="16" t="s">
+      <c r="K2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -952,34 +952,34 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="G3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="I3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="J3" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -987,34 +987,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1022,34 +1022,34 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J5" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1057,34 +1057,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J6" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1092,34 +1092,34 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J7" s="19" t="s">
+      <c r="K7" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1127,34 +1127,34 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J8" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" s="19" t="s">
-        <v>44</v>
-      </c>
       <c r="K8" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1162,34 +1162,34 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" s="18" t="s">
+      <c r="K9" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1197,34 +1197,34 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J10" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="K10" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="J10" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1232,34 +1232,34 @@
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="K11" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J11" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1267,34 +1267,34 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J12" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="K12" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J12" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1302,34 +1302,34 @@
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="K13" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J13" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1337,34 +1337,34 @@
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J14" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="K14" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J14" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.2">
@@ -1372,34 +1372,34 @@
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J15" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J15" s="18" t="s">
-        <v>61</v>
-      </c>
       <c r="K15" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="3" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1407,34 +1407,34 @@
         <v>15</v>
       </c>
       <c r="B16" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="D16" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="E16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="I16" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="J16" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="K16" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="E16" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="F16" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="G16" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="H16" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="I16" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>